<commit_message>
updated on sept 29
</commit_message>
<xml_diff>
--- a/12604000.xlsx
+++ b/12604000.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khush\Desktop\PYTHON\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BCAFAF-0FE3-4F2A-920A-9AC3F654C379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD679D5-65BD-4C5C-84B7-AA86D96A3214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -323,6 +323,9 @@
   </si>
   <si>
     <t>GOOD GOING</t>
+  </si>
+  <si>
+    <t>REST TIME</t>
   </si>
 </sst>
 </file>
@@ -2817,26 +2820,50 @@
       </c>
     </row>
     <row r="43" spans="1:14" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="13"/>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="14" t="str">
+      <c r="A43" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B43" s="15">
+        <v>600</v>
+      </c>
+      <c r="C43" s="15">
+        <v>0</v>
+      </c>
+      <c r="D43" s="15">
+        <v>50</v>
+      </c>
+      <c r="E43" s="15">
+        <v>0</v>
+      </c>
+      <c r="F43" s="15">
+        <v>0</v>
+      </c>
+      <c r="G43" s="15">
+        <v>0</v>
+      </c>
+      <c r="H43" s="15">
+        <v>0</v>
+      </c>
+      <c r="I43" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="14" t="str">
+        <v>650</v>
+      </c>
+      <c r="J43" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
+        <v>790</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="44" spans="1:14" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13"/>

</xml_diff>

<commit_message>
updated on oct 23
</commit_message>
<xml_diff>
--- a/12604000.xlsx
+++ b/12604000.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khush\Desktop\PYTHON\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EED0EE-2673-45A7-A942-6CC6686DBEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D41DD1-5F6E-4133-ACC9-1C17540DDD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="113">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>DAY WENT WELL</t>
+  </si>
+  <si>
+    <t>TRAVELING</t>
   </si>
 </sst>
 </file>
@@ -3647,26 +3650,50 @@
       </c>
     </row>
     <row r="60" spans="1:14" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="13"/>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="15"/>
-      <c r="I60" s="14" t="str">
+      <c r="A60" s="13">
+        <v>46318</v>
+      </c>
+      <c r="B60" s="15">
+        <v>380</v>
+      </c>
+      <c r="C60" s="15">
+        <v>0</v>
+      </c>
+      <c r="D60" s="15">
+        <v>140</v>
+      </c>
+      <c r="E60" s="15">
+        <v>0</v>
+      </c>
+      <c r="F60" s="15">
+        <v>0</v>
+      </c>
+      <c r="G60" s="15">
+        <v>0</v>
+      </c>
+      <c r="H60" s="15">
+        <v>50</v>
+      </c>
+      <c r="I60" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="14" t="str">
+        <v>570</v>
+      </c>
+      <c r="J60" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="17"/>
+        <v>870</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N60" s="17" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="61" spans="1:14" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="13"/>

</xml_diff>